<commit_message>
data: 2026-07-21 일별 수집
</commit_message>
<xml_diff>
--- a/data/daily/2026-07/2026-07-21.xlsx
+++ b/data/daily/2026-07/2026-07-21.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="카카오선물하기" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="다이소몰" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="카테고리통계" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="카카오선물하기" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="다이소몰" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="카테고리통계" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,13 +19,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -36,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -44,12 +47,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -427,32 +439,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>순위</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>상품명</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>브랜드</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>가격</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>상품URL</t>
         </is>
@@ -941,7 +953,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>피부/미용</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -949,29 +961,29 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2입 추가 증정 "선물하기 1등 콜라겐" 아일로 타입1 콜라겐 비오틴 앰플 28일분 오간자 에디션+ 앰플 2입 추가 증정</t>
+          <t>[한끼통살] 닭가슴살 순삭 10팩세트(소스통살5+닭가슴살볼5)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>아일로</t>
+          <t>한끼통살</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>61,900원</t>
+          <t>19,900원</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/4965835</t>
+          <t>https://gift.kakao.com/product/10848340</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>기타/특수목적</t>
+          <t>피부/미용</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -979,29 +991,29 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>[그레인온] 골드 카무트 브랜드밀효소G 3개월분+10포증정(총100포)</t>
+          <t>2입 추가 증정 "선물하기 1등 콜라겐" 아일로 타입1 콜라겐 비오틴 앰플 28일분 오간자 에디션+ 앰플 2입 추가 증정</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>그레인온</t>
+          <t>아일로</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>24,900원</t>
+          <t>61,900원</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/13180362</t>
+          <t>https://gift.kakao.com/product/4965835</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>다이어트/체중관리</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1009,22 +1021,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>[한끼통살] 닭가슴살 순삭 10팩세트(소스통살5+닭가슴살볼5)</t>
+          <t>[그레인온] 골드 카무트 브랜드밀효소G 3개월분+10포증정(총100포)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>한끼통살</t>
+          <t>그레인온</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>19,900원</t>
+          <t>24,900원</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/10848340</t>
+          <t>https://gift.kakao.com/product/13180362</t>
         </is>
       </c>
     </row>
@@ -1081,32 +1093,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>순위</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>상품명</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>브랜드</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>가격</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>상품URL</t>
         </is>
@@ -1123,29 +1135,29 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>녹차 카테킨 6정 6일분</t>
+          <t>[신혜선 PICK] 동국 마이팝 푸룬＆식이섬유</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>대웅제약</t>
+          <t>동국제약</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1,000원</t>
+          <t>2,000원</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000282&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=610911029&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>멀티비타민/종합비타민</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -1153,29 +1165,29 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>멀티비타민 미네랄 츄어블 60정 30일분</t>
+          <t>[신혜선 PICK] 동국 마이팝 발효효소＆매실</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>대웅제약</t>
+          <t>동국제약</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>5,000원</t>
+          <t>2,000원</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000142&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=610911031&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>기타/특수목적</t>
+          <t>프로바이오틱스/유산균</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -1183,7 +1195,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>[신혜선 PICK] 동국 마이팝 푸룬＆식이섬유</t>
+          <t>이너케어＆유산균 30캡슐</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1193,19 +1205,19 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2,000원</t>
+          <t>5,000원</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=610911029&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=610910677&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>혈행</t>
+          <t>마그네슘</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -1213,7 +1225,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>코엔자임 Q10 30캡슐 30일분</t>
+          <t>마그네슘 30정 30일분</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1223,19 +1235,19 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>5,000원</t>
+          <t>3,000원</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000144&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000128&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>기타/특수목적</t>
+          <t>비타민D</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -1243,22 +1255,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>하루한포 쌍화차 5포 5일분</t>
+          <t>비타민D 4000IU 30정 30일분</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>휴럼</t>
+          <t>대웅제약</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2,000원</t>
+          <t>3,000원</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=919157055&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000132&amp;recmYn=N</t>
         </is>
       </c>
     </row>
@@ -1273,29 +1285,29 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>하루한포 유기농 컬리케일 15포 15일분</t>
+          <t>동국 맛있는 센시안 브이캔디 20정 20일분</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>휴럼</t>
+          <t>동국제약</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5,000원</t>
+          <t>3,000원</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=919157057&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=610910968&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>프로바이오틱스/유산균</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -1303,12 +1315,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>이너케어＆유산균 30캡슐</t>
+          <t>콜린 미오이노시톨 4000 10포</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>동국제약</t>
+          <t>안국약품</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1318,7 +1330,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=610910677&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=985472642&amp;recmYn=N</t>
         </is>
       </c>
     </row>
@@ -1333,22 +1345,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>영진 리얼바몬드 비타C 1500</t>
+          <t>데일리와이즈 푸룬 구미 7일분</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>영진약품</t>
+          <t>종근당</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>5,000원</t>
+          <t>1,000원</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=034507002&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=032306208&amp;recmYn=N</t>
         </is>
       </c>
     </row>
@@ -1363,12 +1375,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>정성담은 배도라지스틱 12포</t>
+          <t>하루한포 유기농 야채분말 15포 15일분</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>자연관</t>
+          <t>휴럼</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1378,14 +1390,14 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=901762093&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=919157056&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>피부/미용</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -1393,22 +1405,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>마데카 저분자 콜라겐C</t>
+          <t>바나바잎 추출물 30정 (30일분)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>동국제약</t>
+          <t>대웅제약</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>5,000원</t>
+          <t>3,000원</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=610910603&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000131&amp;recmYn=N</t>
         </is>
       </c>
     </row>
@@ -1435,32 +1447,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>전체</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>비율(%)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>카카오선물하기</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>다이소몰</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>올리브영</t>
         </is>
@@ -1473,16 +1485,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>30</v>
+        <v>26.7</v>
       </c>
       <c r="D2" t="n">
         <v>8</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -1517,16 +1529,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>3.3</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -1539,16 +1551,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>3.3</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -1583,16 +1595,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>3.3</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -1627,16 +1639,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C9" t="n">
-        <v>13.3</v>
+        <v>16.7</v>
       </c>
       <c r="D9" t="n">
         <v>4</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
@@ -1671,16 +1683,16 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C11" t="n">
-        <v>6.7</v>
+        <v>3.3</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
올리브영 수동 입력 (2026-07-21, 2026-07-22, 캡쳐 기반 TOP10)
Turnstile 차단으로 캡쳐 이미지에서 TOP10 추출해 반영, 카테고리통계 재계산
</commit_message>
<xml_diff>
--- a/data/daily/2026-07/2026-07-21.xlsx
+++ b/data/daily/2026-07/2026-07-21.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="카카오선물하기" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="다이소몰" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="카테고리통계" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="카카오선물하기" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="다이소몰" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="카테고리통계" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="올리브영" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1447,32 +1448,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>전체</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>비율(%)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>카카오선물하기</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>다이소몰</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>올리브영</t>
         </is>
@@ -1488,7 +1489,7 @@
         <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>26.7</v>
+        <v>20</v>
       </c>
       <c r="D2" t="n">
         <v>8</v>
@@ -1507,10 +1508,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -1519,7 +1520,7 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -1532,7 +1533,7 @@
         <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>3.3</v>
+        <v>2.5</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -1554,7 +1555,7 @@
         <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>3.3</v>
+        <v>2.5</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -1620,7 +1621,7 @@
         <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>3.3</v>
+        <v>2.5</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
@@ -1639,10 +1640,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C9" t="n">
-        <v>16.7</v>
+        <v>15</v>
       </c>
       <c r="D9" t="n">
         <v>4</v>
@@ -1651,7 +1652,7 @@
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -1661,10 +1662,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C10" t="n">
-        <v>3.3</v>
+        <v>12.5</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -1673,7 +1674,7 @@
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -1683,10 +1684,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C11" t="n">
-        <v>3.3</v>
+        <v>5</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
@@ -1695,7 +1696,7 @@
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -1705,10 +1706,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C12" t="n">
-        <v>40</v>
+        <v>37.5</v>
       </c>
       <c r="D12" t="n">
         <v>6</v>
@@ -1717,7 +1718,7 @@
         <v>6</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -1727,7 +1728,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C13" t="n">
         <v>100</v>
@@ -1739,8 +1740,322 @@
         <v>10</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
-      </c>
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>카테고리</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>순위</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>상품명</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>가격</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>상품URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>프로바이오틱스/유산균</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>비비랩 슬림 밸런스 유산균 2g x 30포 (15일분)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>비비랩</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>18,900원</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>프로바이오틱스/유산균</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>비비랩 데일리 밸런스 유산균 2g x 30포 (1개월분)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>비비랩</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>16,900원</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>다이어트/체중관리</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>프로뉴트리션 듀얼플랜 다이어트 유산균 14포</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>프로뉴트리션</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>35,800원</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>피부/미용</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>[7월 올영픽/단독기획] 비비랩 저분자콜라겐S 30포 단품/더블기획</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>비비랩</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>26,900원</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>비타민C/항산화</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>고려은단 비타민C1000 600정 (20개월분)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>고려은단</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>42,900원</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>기타/특수목적</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>[7월 올영픽] 콜레올로직 컷팅 젤리 레몬/키위/석류 10+2+2포 기획</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>푸드올로지</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>18,800원</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>기타/특수목적</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>올더베리 웰니스 구미 30일분 6종 택1</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>올더베리</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>9,500원</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>기타/특수목적</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>[골라담기] CJ웰케어 건강루틴 10종 택1 가격혁명</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>씨제이웰케어</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>5,900원</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>프로바이오틱스/유산균</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>[올영단독] 지노마스터 질유산균 70캡슐 (70일분)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>지노마스터</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>59,000원</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>프로바이오틱스/유산균</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>[덴프스] 덴마크 유산균이야기 우먼 2개월분(질유산균)+철분 헤모케어3</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>덴프스</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>39,000원</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>